<commit_message>
add start date and starting additional data code
</commit_message>
<xml_diff>
--- a/balance_generate/input_data/bank_data_only_dep.xlsx
+++ b/balance_generate/input_data/bank_data_only_dep.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dzimi\Documents\data_engineering\data_projects\git_hub_projects\bank_project\balance_generate\input_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{889729A8-AE6F-417D-BD74-7670CC59D47B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A68D213-1690-4E3F-8645-656C916C1163}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -818,7 +818,7 @@
         <v>1</v>
       </c>
       <c r="D9">
-        <v>7000</v>
+        <v>7060</v>
       </c>
       <c r="E9" t="s">
         <v>25</v>

</xml_diff>

<commit_message>
add variables for mortgages, starting sql with curves
</commit_message>
<xml_diff>
--- a/balance_generate/input_data/bank_data_only_dep.xlsx
+++ b/balance_generate/input_data/bank_data_only_dep.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dzimi\Documents\data_engineering\data_projects\git_hub_projects\bank_project\balance_generate\input_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A68D213-1690-4E3F-8645-656C916C1163}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{984F6ED0-3776-4489-A0D0-DBB15D601487}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-1425" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="bs_structure" sheetId="2" r:id="rId1"/>
@@ -494,6 +494,7 @@
     <col min="6" max="6" width="20.1796875" customWidth="1"/>
     <col min="7" max="7" width="14" customWidth="1"/>
     <col min="10" max="10" width="12.81640625" customWidth="1"/>
+    <col min="12" max="12" width="10.1796875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="12.81640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -561,7 +562,7 @@
         <v>4</v>
       </c>
       <c r="H2" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="I2" t="s">
         <v>39</v>
@@ -678,7 +679,7 @@
         <v>4</v>
       </c>
       <c r="H5" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="I5" t="s">
         <v>16</v>

</xml_diff>

<commit_message>
finish curve gemeration and fixings tables
</commit_message>
<xml_diff>
--- a/balance_generate/input_data/bank_data_only_dep.xlsx
+++ b/balance_generate/input_data/bank_data_only_dep.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dzimi\Documents\data_engineering\data_projects\git_hub_projects\bank_project\balance_generate\input_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E432D553-C8CF-4778-8C21-3D433E76CB2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{756B3CD2-EB74-4719-A450-AB2AEBE08F9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1040" yWindow="1130" windowWidth="21600" windowHeight="11180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1280" yWindow="4150" windowWidth="21600" windowHeight="11180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="bs_structure" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="48">
   <si>
     <t>A</t>
   </si>
@@ -168,6 +168,18 @@
   </si>
   <si>
     <t>WIB7Y</t>
+  </si>
+  <si>
+    <t>disc_curve</t>
+  </si>
+  <si>
+    <t>fwd_curve</t>
+  </si>
+  <si>
+    <t>PLN_disc_curve</t>
+  </si>
+  <si>
+    <t>PLN_fwd_curve</t>
   </si>
 </sst>
 </file>
@@ -486,7 +498,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8188D07C-A870-4194-AE82-5ADE66722983}">
-  <dimension ref="A1:M14"/>
+  <dimension ref="A1:O14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.6328125" customWidth="1"/>
@@ -499,9 +511,11 @@
     <col min="10" max="10" width="12.81640625" customWidth="1"/>
     <col min="12" max="12" width="10.1796875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="12.81640625" customWidth="1"/>
+    <col min="14" max="14" width="17.7265625" customWidth="1"/>
+    <col min="15" max="15" width="13.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>23</v>
       </c>
@@ -541,8 +555,14 @@
       <c r="M1" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N1" t="s">
+        <v>44</v>
+      </c>
+      <c r="O1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>45657</v>
       </c>
@@ -582,8 +602,14 @@
       <c r="M2" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N2" t="s">
+        <v>46</v>
+      </c>
+      <c r="O2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>45657</v>
       </c>
@@ -623,8 +649,14 @@
       <c r="M3" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N3" t="s">
+        <v>46</v>
+      </c>
+      <c r="O3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
         <v>45657</v>
       </c>
@@ -661,8 +693,14 @@
       <c r="M4" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N4" t="s">
+        <v>46</v>
+      </c>
+      <c r="O4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>45657</v>
       </c>
@@ -702,8 +740,14 @@
       <c r="M5" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N5" t="s">
+        <v>46</v>
+      </c>
+      <c r="O5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
         <v>45657</v>
       </c>
@@ -743,8 +787,14 @@
       <c r="M6" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N6" t="s">
+        <v>46</v>
+      </c>
+      <c r="O6" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>45657</v>
       </c>
@@ -781,8 +831,14 @@
       <c r="M7" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N7" t="s">
+        <v>46</v>
+      </c>
+      <c r="O7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
         <v>45657</v>
       </c>
@@ -822,8 +878,14 @@
       <c r="M8" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N8" t="s">
+        <v>46</v>
+      </c>
+      <c r="O8" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A9" s="1">
         <v>45657</v>
       </c>
@@ -854,8 +916,14 @@
       <c r="K9" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N9" t="s">
+        <v>46</v>
+      </c>
+      <c r="O9" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A10" s="1">
         <v>45657</v>
       </c>
@@ -886,8 +954,14 @@
       <c r="K10" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N10" t="s">
+        <v>46</v>
+      </c>
+      <c r="O10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A11" s="1">
         <v>45657</v>
       </c>
@@ -918,8 +992,14 @@
       <c r="K11" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N11" t="s">
+        <v>46</v>
+      </c>
+      <c r="O11" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A12" s="1">
         <v>45657</v>
       </c>
@@ -944,8 +1024,14 @@
       <c r="I12" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N12" t="s">
+        <v>46</v>
+      </c>
+      <c r="O12" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A13" s="1">
         <v>45657</v>
       </c>
@@ -976,8 +1062,14 @@
       <c r="K13" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N13" t="s">
+        <v>46</v>
+      </c>
+      <c r="O13" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A14" s="1">
         <v>45657</v>
       </c>
@@ -1007,6 +1099,12 @@
       </c>
       <c r="K14" t="s">
         <v>20</v>
+      </c>
+      <c r="N14" t="s">
+        <v>46</v>
+      </c>
+      <c r="O14" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
sched id tables added
</commit_message>
<xml_diff>
--- a/balance_generate/input_data/bank_data_only_dep.xlsx
+++ b/balance_generate/input_data/bank_data_only_dep.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dzimi\Documents\data_engineering\data_projects\git_hub_projects\bank_project\balance_generate\input_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{756B3CD2-EB74-4719-A450-AB2AEBE08F9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C50ECB54-3A9C-4317-8CFE-20248E081C48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1280" yWindow="4150" windowWidth="21600" windowHeight="11180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="bs_structure" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="52">
   <si>
     <t>A</t>
   </si>
@@ -180,16 +180,34 @@
   </si>
   <si>
     <t>PLN_fwd_curve</t>
+  </si>
+  <si>
+    <t>basis</t>
+  </si>
+  <si>
+    <t>b_day_conv</t>
+  </si>
+  <si>
+    <t>ModifiedFollowing</t>
+  </si>
+  <si>
+    <t>ACT/365</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -498,7 +516,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8188D07C-A870-4194-AE82-5ADE66722983}">
-  <dimension ref="A1:O14"/>
+  <dimension ref="A1:Q14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.6328125" customWidth="1"/>
@@ -510,12 +528,12 @@
     <col min="7" max="7" width="14" customWidth="1"/>
     <col min="10" max="10" width="12.81640625" customWidth="1"/>
     <col min="12" max="12" width="10.1796875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.81640625" customWidth="1"/>
-    <col min="14" max="14" width="17.7265625" customWidth="1"/>
-    <col min="15" max="15" width="13.7265625" bestFit="1" customWidth="1"/>
+    <col min="13" max="15" width="12.81640625" customWidth="1"/>
+    <col min="16" max="16" width="17.7265625" customWidth="1"/>
+    <col min="17" max="17" width="13.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>23</v>
       </c>
@@ -556,13 +574,19 @@
         <v>32</v>
       </c>
       <c r="N1" t="s">
+        <v>48</v>
+      </c>
+      <c r="O1" t="s">
+        <v>49</v>
+      </c>
+      <c r="P1" t="s">
         <v>44</v>
       </c>
-      <c r="O1" t="s">
+      <c r="Q1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>45657</v>
       </c>
@@ -603,13 +627,19 @@
         <v>38</v>
       </c>
       <c r="N2" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="O2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
+        <v>50</v>
+      </c>
+      <c r="P2" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>45657</v>
       </c>
@@ -650,13 +680,19 @@
         <v>10</v>
       </c>
       <c r="N3" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="O3" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
+        <v>50</v>
+      </c>
+      <c r="P3" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
         <v>45657</v>
       </c>
@@ -694,13 +730,19 @@
         <v>43</v>
       </c>
       <c r="N4" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="O4" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
+        <v>50</v>
+      </c>
+      <c r="P4" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>45657</v>
       </c>
@@ -741,13 +783,19 @@
         <v>10</v>
       </c>
       <c r="N5" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="O5" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
+        <v>50</v>
+      </c>
+      <c r="P5" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
         <v>45657</v>
       </c>
@@ -788,13 +836,19 @@
         <v>10</v>
       </c>
       <c r="N6" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="O6" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
+        <v>50</v>
+      </c>
+      <c r="P6" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>45657</v>
       </c>
@@ -832,13 +886,19 @@
         <v>38</v>
       </c>
       <c r="N7" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="O7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
+        <v>50</v>
+      </c>
+      <c r="P7" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
         <v>45657</v>
       </c>
@@ -879,13 +939,19 @@
         <v>40</v>
       </c>
       <c r="N8" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="O8" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
+        <v>50</v>
+      </c>
+      <c r="P8" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A9" s="1">
         <v>45657</v>
       </c>
@@ -917,13 +983,19 @@
         <v>17</v>
       </c>
       <c r="N9" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="O9" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
+        <v>50</v>
+      </c>
+      <c r="P9" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A10" s="1">
         <v>45657</v>
       </c>
@@ -955,13 +1027,19 @@
         <v>19</v>
       </c>
       <c r="N10" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="O10" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
+        <v>50</v>
+      </c>
+      <c r="P10" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A11" s="1">
         <v>45657</v>
       </c>
@@ -993,13 +1071,19 @@
         <v>19</v>
       </c>
       <c r="N11" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="O11" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
+        <v>50</v>
+      </c>
+      <c r="P11" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A12" s="1">
         <v>45657</v>
       </c>
@@ -1024,14 +1108,14 @@
       <c r="I12" t="s">
         <v>18</v>
       </c>
-      <c r="N12" t="s">
-        <v>46</v>
-      </c>
-      <c r="O12" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P12" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A13" s="1">
         <v>45657</v>
       </c>
@@ -1062,14 +1146,14 @@
       <c r="K13" t="s">
         <v>20</v>
       </c>
-      <c r="N13" t="s">
-        <v>46</v>
-      </c>
-      <c r="O13" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P13" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A14" s="1">
         <v>45657</v>
       </c>
@@ -1100,14 +1184,15 @@
       <c r="K14" t="s">
         <v>20</v>
       </c>
-      <c r="N14" t="s">
-        <v>46</v>
-      </c>
-      <c r="O14" t="s">
+      <c r="P14" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q14" t="s">
         <v>47</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
building cash flow and some repair in previuos steps
</commit_message>
<xml_diff>
--- a/balance_generate/input_data/bank_data_only_dep.xlsx
+++ b/balance_generate/input_data/bank_data_only_dep.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dzimi\Documents\data_engineering\data_projects\git_hub_projects\bank_project\balance_generate\input_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C50ECB54-3A9C-4317-8CFE-20248E081C48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDEDF0EC-A685-4B08-ABBC-4397508403D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-1425" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="bs_structure" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="53">
   <si>
     <t>A</t>
   </si>
@@ -68,9 +68,6 @@
     <t>30Y</t>
   </si>
   <si>
-    <t>WIB3M</t>
-  </si>
-  <si>
     <t>current_account</t>
   </si>
   <si>
@@ -152,24 +149,15 @@
     <t>3M</t>
   </si>
   <si>
-    <t>WIB5Y</t>
-  </si>
-  <si>
     <t>25Y</t>
   </si>
   <si>
-    <t>WIB6M</t>
-  </si>
-  <si>
     <t>investment_loan_float</t>
   </si>
   <si>
     <t>retained_earnings</t>
   </si>
   <si>
-    <t>WIB7Y</t>
-  </si>
-  <si>
     <t>disc_curve</t>
   </si>
   <si>
@@ -182,9 +170,6 @@
     <t>PLN_fwd_curve</t>
   </si>
   <si>
-    <t>basis</t>
-  </si>
-  <si>
     <t>b_day_conv</t>
   </si>
   <si>
@@ -192,6 +177,24 @@
   </si>
   <si>
     <t>ACT/365</t>
+  </si>
+  <si>
+    <t>dc_conv</t>
+  </si>
+  <si>
+    <t>PLN_ASK_5Y</t>
+  </si>
+  <si>
+    <t>PLN_ASK_3M</t>
+  </si>
+  <si>
+    <t>PLN_ASK_7Y</t>
+  </si>
+  <si>
+    <t>PLN_ASK_6M</t>
+  </si>
+  <si>
+    <t>PLN_BID_6M</t>
   </si>
 </sst>
 </file>
@@ -535,31 +538,31 @@
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1" t="s">
         <v>23</v>
       </c>
-      <c r="B1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C1" t="s">
-        <v>24</v>
-      </c>
       <c r="D1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H1" t="s">
         <v>3</v>
       </c>
       <c r="I1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J1" t="s">
         <v>4</v>
@@ -571,19 +574,19 @@
         <v>6</v>
       </c>
       <c r="M1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="N1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="O1" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="P1" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="Q1" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.35">
@@ -600,7 +603,7 @@
         <v>1000</v>
       </c>
       <c r="E2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F2" t="s">
         <v>7</v>
@@ -609,34 +612,34 @@
         <v>4</v>
       </c>
       <c r="H2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="J2">
         <v>1</v>
       </c>
       <c r="K2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="L2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="M2" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="N2" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="O2" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="P2" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="Q2" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.35">
@@ -653,7 +656,7 @@
         <v>1100</v>
       </c>
       <c r="E3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F3" t="s">
         <v>7</v>
@@ -671,25 +674,25 @@
         <v>1</v>
       </c>
       <c r="K3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="L3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="M3" t="s">
-        <v>10</v>
+        <v>49</v>
       </c>
       <c r="N3" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="O3" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="P3" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="Q3" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.35">
@@ -706,7 +709,7 @@
         <v>2000</v>
       </c>
       <c r="E4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F4" t="s">
         <v>7</v>
@@ -715,31 +718,31 @@
         <v>4</v>
       </c>
       <c r="H4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J4">
         <v>1</v>
       </c>
       <c r="K4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="M4" t="s">
+        <v>50</v>
+      </c>
+      <c r="N4" t="s">
+        <v>46</v>
+      </c>
+      <c r="O4" t="s">
+        <v>45</v>
+      </c>
+      <c r="P4" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q4" t="s">
         <v>43</v>
-      </c>
-      <c r="N4" t="s">
-        <v>51</v>
-      </c>
-      <c r="O4" t="s">
-        <v>50</v>
-      </c>
-      <c r="P4" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.35">
@@ -756,7 +759,7 @@
         <v>2100</v>
       </c>
       <c r="E5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F5" t="s">
         <v>7</v>
@@ -768,31 +771,31 @@
         <v>8</v>
       </c>
       <c r="I5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J5">
         <v>1</v>
       </c>
       <c r="K5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="L5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="M5" t="s">
-        <v>10</v>
+        <v>49</v>
       </c>
       <c r="N5" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="O5" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="P5" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="Q5" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.35">
@@ -809,7 +812,7 @@
         <v>4100</v>
       </c>
       <c r="E6" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="F6" t="s">
         <v>7</v>
@@ -821,31 +824,31 @@
         <v>8</v>
       </c>
       <c r="I6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="L6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="M6" t="s">
-        <v>10</v>
+        <v>49</v>
       </c>
       <c r="N6" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="O6" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="P6" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="Q6" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.35">
@@ -862,7 +865,7 @@
         <v>3000</v>
       </c>
       <c r="E7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F7" t="s">
         <v>7</v>
@@ -871,31 +874,31 @@
         <v>1</v>
       </c>
       <c r="H7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="M7" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="N7" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="O7" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="P7" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="Q7" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.35">
@@ -912,7 +915,7 @@
         <v>3100</v>
       </c>
       <c r="E8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F8" t="s">
         <v>7</v>
@@ -924,31 +927,31 @@
         <v>8</v>
       </c>
       <c r="I8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="L8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="M8" t="s">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="N8" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="O8" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="P8" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="Q8" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.35">
@@ -965,7 +968,7 @@
         <v>7060</v>
       </c>
       <c r="E9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F9" t="s">
         <v>7</v>
@@ -974,25 +977,28 @@
         <v>4</v>
       </c>
       <c r="H9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K9" t="s">
-        <v>17</v>
+        <v>16</v>
+      </c>
+      <c r="M9" t="s">
+        <v>52</v>
       </c>
       <c r="N9" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="O9" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="P9" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="Q9" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.35">
@@ -1009,7 +1015,7 @@
         <v>6000</v>
       </c>
       <c r="E10" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F10" t="s">
         <v>7</v>
@@ -1021,22 +1027,22 @@
         <v>0</v>
       </c>
       <c r="I10" t="s">
+        <v>17</v>
+      </c>
+      <c r="K10" t="s">
         <v>18</v>
       </c>
-      <c r="K10" t="s">
-        <v>19</v>
-      </c>
       <c r="N10" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="O10" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="P10" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="Q10" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.35">
@@ -1053,7 +1059,7 @@
         <v>8000</v>
       </c>
       <c r="E11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F11" t="s">
         <v>7</v>
@@ -1065,22 +1071,22 @@
         <v>0</v>
       </c>
       <c r="I11" t="s">
+        <v>17</v>
+      </c>
+      <c r="K11" t="s">
         <v>18</v>
       </c>
-      <c r="K11" t="s">
-        <v>19</v>
-      </c>
       <c r="N11" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="O11" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="P11" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="Q11" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.35">
@@ -1097,7 +1103,7 @@
         <v>5000</v>
       </c>
       <c r="E12" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F12" t="s">
         <v>7</v>
@@ -1106,13 +1112,13 @@
         <v>14</v>
       </c>
       <c r="I12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="P12" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="Q12" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.35">
@@ -1129,7 +1135,7 @@
         <v>5001</v>
       </c>
       <c r="E13" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F13" t="s">
         <v>7</v>
@@ -1138,19 +1144,19 @@
         <v>8</v>
       </c>
       <c r="H13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="K13" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="P13" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="Q13" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.35">
@@ -1167,7 +1173,7 @@
         <v>5002</v>
       </c>
       <c r="E14" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F14" t="s">
         <v>7</v>
@@ -1176,19 +1182,19 @@
         <v>8</v>
       </c>
       <c r="H14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="K14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="P14" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="Q14" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>